<commit_message>
UI improvements and documentation update (v2.4.1)
- Remove Display Settings UI, set plot width to Full by default
- Move Fit Results table from control panel to below spectrum plot
- Remove overlapping Residuals subplot title
- Rewrite COMPLETION_SUMMARY.md to reflect current v2.4.0+ state
- Update CHANGELOG.md with v2.4.1 entry
- Add USER_GUIDE.md, start.bat, start.sh

Co-Authored-By: Claude Opus 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SpectralFit/presets/material_presets.xlsx
+++ b/SpectralFit/presets/material_presets.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29721"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="60" documentId="11_964FAD5F4877018EBB05B99852E61E51D59031B2" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3C44FB98-347F-4477-A122-46AC12631109}"/>
+  <xr:revisionPtr revIDLastSave="67" documentId="11_964FAD5F4877018EBB05B99852E61E51D59031B2" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A6684A15-CADB-4A0B-97F8-1B680A3AB9E5}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="WSe2_PL" sheetId="5" r:id="rId1"/>
@@ -684,7 +684,7 @@
         <v>200</v>
       </c>
       <c r="C2">
-        <v>400</v>
+        <v>350</v>
       </c>
       <c r="D2">
         <v>8</v>
@@ -736,10 +736,10 @@
         <v>10</v>
       </c>
       <c r="D5">
-        <v>10000</v>
+        <v>500</v>
       </c>
       <c r="E5">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F5">
         <v>0.3</v>
@@ -759,10 +759,10 @@
         <v>10</v>
       </c>
       <c r="D6">
-        <v>12000</v>
+        <v>200</v>
       </c>
       <c r="E6">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="F6">
         <v>0.3</v>
@@ -782,10 +782,10 @@
         <v>10</v>
       </c>
       <c r="D7">
-        <v>12000</v>
+        <v>200</v>
       </c>
       <c r="E7">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F7">
         <v>0.3</v>

</xml_diff>

<commit_message>
Multi-select file picker, raw row at top of PL fit results (v2.5.0)
Replaces the folder-picker entry point with a native OS multi-select
file dialog (askopenfilenames), JSON-serialized across the subprocess
boundary so paths with spaces/commas/unicode survive intact. Last-picked
directory is remembered; cancel is a clean no-op; re-picked files are
skipped silently. Multi-Y splitting, mode auto-detection, and per-file
error isolation are preserved.

Also reorders the PL "Raw" summary row to the top of the fit-results
table and the exported master CSV for easier raw-vs-fit comparison.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SpectralFit/presets/material_presets.xlsx
+++ b/SpectralFit/presets/material_presets.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29721"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30110"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="67" documentId="11_964FAD5F4877018EBB05B99852E61E51D59031B2" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A6684A15-CADB-4A0B-97F8-1B680A3AB9E5}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_7E436F5E4A6213BD00241E96FF5300FE471BA61C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5B969BDA-24AC-4BE9-9C72-3DF62D91C11E}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="WSe2_PL" sheetId="5" r:id="rId1"/>
-    <sheet name="WSe2_Raman" sheetId="4" r:id="rId2"/>
-    <sheet name="MoS2_Raman" sheetId="2" r:id="rId3"/>
-    <sheet name="Silicon_Raman" sheetId="3" r:id="rId4"/>
+    <sheet name="WSe2_PL" sheetId="1" r:id="rId1"/>
+    <sheet name="WSe2_Raman" sheetId="2" r:id="rId2"/>
+    <sheet name="MoS2_Raman" sheetId="3" r:id="rId3"/>
+    <sheet name="Silicon_Raman" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -500,7 +500,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{339DF148-B2DF-443A-B9D6-3B434E8B7DB6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -590,16 +590,16 @@
         <v>20</v>
       </c>
       <c r="B5">
-        <v>750</v>
+        <v>770</v>
       </c>
       <c r="C5">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="D5">
         <v>1000</v>
       </c>
       <c r="E5">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="F5">
         <v>0.3</v>
@@ -613,16 +613,16 @@
         <v>22</v>
       </c>
       <c r="B6">
-        <v>780</v>
+        <v>800</v>
       </c>
       <c r="C6">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="D6">
         <v>200</v>
       </c>
       <c r="E6">
-        <v>80</v>
+        <v>50</v>
       </c>
       <c r="F6">
         <v>0.3</v>
@@ -637,7 +637,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{13D7C7CD-749B-4620-A10F-D7F969539AAC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:J7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -800,7 +800,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:J6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -937,7 +937,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:J5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
Add "Delete All Files" button; bump to v2.6.0
@
- Sidebar: new "Delete All Files" button in the "Loaded Files" section,
  next to "Remove File" (two-column layout), wired to the existing
  clear_all_files() helper. One click clears all loaded spectra.
- Bump version 2.5.0 -> 2.6.0 across CHANGELOG, README, and Summary.
- Also includes a pre-existing baseline-preview fix in control_panel.py
  (preview now runs even after a fit exists) and an updated
  material_presets.xlsx.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
@
</commit_message>
<xml_diff>
--- a/SpectralFit/presets/material_presets.xlsx
+++ b/SpectralFit/presets/material_presets.xlsx
@@ -1,11 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30125"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_7E436F5E4A6213BD00241E96FF5300FE471BA61C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5B969BDA-24AC-4BE9-9C72-3DF62D91C11E}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nexstrom-my.sharepoint.com/personal/angyu_lu_nexstrom_com/Documents/NS/Data/Raman_PL/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="81" documentId="11_7E436F5E4A6213BD00241E96FF5300FE471BA61C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{40E956F4-98C4-4032-94BE-941B71412823}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="WSe2_PL" sheetId="1" r:id="rId1"/>
@@ -34,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="45">
   <si>
     <t>x_range_enabled</t>
   </si>
@@ -69,7 +74,7 @@
     <t>ALS</t>
   </si>
   <si>
-    <t>650-900</t>
+    <t>650-880</t>
   </si>
   <si>
     <t>WSe2 PL peaks</t>
@@ -108,22 +113,52 @@
     <t>#9467bd</t>
   </si>
   <si>
-    <t>WSe2 E2g and 2LA peaks</t>
+    <t>WSe2 Raman</t>
+  </si>
+  <si>
+    <t>E2g+A1g</t>
+  </si>
+  <si>
+    <t>#EF482E</t>
+  </si>
+  <si>
+    <t>2LA</t>
+  </si>
+  <si>
+    <t>#D5EF2E</t>
+  </si>
+  <si>
+    <t>B2g</t>
+  </si>
+  <si>
+    <t>#2ED5EF</t>
+  </si>
+  <si>
+    <t>LB</t>
+  </si>
+  <si>
+    <t>#482EEF</t>
+  </si>
+  <si>
+    <t>LA</t>
+  </si>
+  <si>
+    <t>#76EC32</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>#3276EC</t>
+  </si>
+  <si>
+    <t>375-390; 400-415</t>
+  </si>
+  <si>
+    <t>MoS2 E2g and A1g peaks</t>
   </si>
   <si>
     <t>E2g</t>
-  </si>
-  <si>
-    <t>2LA</t>
-  </si>
-  <si>
-    <t>B2g</t>
-  </si>
-  <si>
-    <t>375-390; 400-415</t>
-  </si>
-  <si>
-    <t>MoS2 E2g and A1g peaks</t>
   </si>
   <si>
     <t>A1g</t>
@@ -502,7 +537,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="10" width="18" customWidth="1"/>
   </cols>
@@ -638,8 +673,8 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:J7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:J11"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="10" width="18" customWidth="1"/>
   </cols>
@@ -681,10 +716,10 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>200</v>
+        <v>-5</v>
       </c>
       <c r="C2">
-        <v>350</v>
+        <v>400</v>
       </c>
       <c r="D2">
         <v>8</v>
@@ -730,50 +765,50 @@
         <v>25</v>
       </c>
       <c r="B5">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="C5">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D5">
         <v>500</v>
       </c>
       <c r="E5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F5">
         <v>0.3</v>
       </c>
       <c r="G5" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B6">
         <v>260</v>
       </c>
       <c r="C6">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D6">
         <v>200</v>
       </c>
       <c r="E6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F6">
         <v>0.3</v>
       </c>
       <c r="G6" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:10">
       <c r="A7" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B7">
         <v>310</v>
@@ -785,13 +820,93 @@
         <v>200</v>
       </c>
       <c r="E7">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="F7">
         <v>0.3</v>
       </c>
       <c r="G7" t="s">
-        <v>23</v>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10">
+      <c r="A8" t="s">
+        <v>31</v>
+      </c>
+      <c r="B8">
+        <v>30</v>
+      </c>
+      <c r="C8">
+        <v>5</v>
+      </c>
+      <c r="E8">
+        <v>2</v>
+      </c>
+      <c r="F8">
+        <v>0.3</v>
+      </c>
+      <c r="G8" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10">
+      <c r="A9" t="s">
+        <v>33</v>
+      </c>
+      <c r="B9">
+        <v>135</v>
+      </c>
+      <c r="C9">
+        <v>10</v>
+      </c>
+      <c r="E9">
+        <v>15</v>
+      </c>
+      <c r="F9">
+        <v>0.3</v>
+      </c>
+      <c r="G9" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10">
+      <c r="A10" t="s">
+        <v>35</v>
+      </c>
+      <c r="B10">
+        <v>17</v>
+      </c>
+      <c r="C10">
+        <v>5</v>
+      </c>
+      <c r="E10">
+        <v>5</v>
+      </c>
+      <c r="F10">
+        <v>0.3</v>
+      </c>
+      <c r="G10" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10">
+      <c r="A11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11">
+        <v>0</v>
+      </c>
+      <c r="C11">
+        <v>3</v>
+      </c>
+      <c r="E11">
+        <v>5</v>
+      </c>
+      <c r="F11">
+        <v>0.3</v>
+      </c>
+      <c r="G11" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -802,7 +917,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:J6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="10" width="18" customWidth="1"/>
   </cols>
@@ -856,10 +971,10 @@
         <v>0.01</v>
       </c>
       <c r="I2" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="J2" t="s">
-        <v>29</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -887,7 +1002,7 @@
     </row>
     <row r="5" spans="1:10">
       <c r="A5" t="s">
-        <v>25</v>
+        <v>39</v>
       </c>
       <c r="B5">
         <v>383</v>
@@ -910,7 +1025,7 @@
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="B6">
         <v>408</v>
@@ -939,7 +1054,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:J5"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="10" width="18" customWidth="1"/>
   </cols>
@@ -984,13 +1099,13 @@
         <v>6</v>
       </c>
       <c r="E2" t="s">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="F2">
         <v>5</v>
       </c>
       <c r="J2" t="s">
-        <v>32</v>
+        <v>42</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -1018,7 +1133,7 @@
     </row>
     <row r="5" spans="1:10">
       <c r="A5" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="B5">
         <v>520</v>
@@ -1036,7 +1151,7 @@
         <v>0.2</v>
       </c>
       <c r="G5" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>